<commit_message>
improved the non metadata feature search
</commit_message>
<xml_diff>
--- a/listings.xlsx
+++ b/listings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\Desktop\Techtics Work\June 2026\TrailerPlace\New Prompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30D20E5-F0C2-47B0-88D2-00085B8188D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2839BF80-5A87-4526-A1B3-4B79D5655030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="listings" sheetId="1" r:id="rId1"/>
@@ -5341,7 +5341,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:P257"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5411,7 +5410,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -5511,7 +5510,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -5561,7 +5560,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -5593,7 +5592,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>66</v>
       </c>
@@ -5625,7 +5624,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>71</v>
       </c>
@@ -5657,7 +5656,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -5689,7 +5688,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -5721,7 +5720,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>91</v>
       </c>
@@ -5753,7 +5752,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>97</v>
       </c>
@@ -5785,7 +5784,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>101</v>
       </c>
@@ -5817,7 +5816,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>107</v>
       </c>
@@ -5849,7 +5848,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -6009,7 +6008,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>134</v>
       </c>
@@ -6059,7 +6058,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>141</v>
       </c>
@@ -6241,7 +6240,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>165</v>
       </c>
@@ -6291,7 +6290,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>174</v>
       </c>
@@ -6323,7 +6322,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>179</v>
       </c>
@@ -6352,7 +6351,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>185</v>
       </c>
@@ -6402,7 +6401,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>196</v>
       </c>
@@ -6434,7 +6433,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>203</v>
       </c>
@@ -6466,7 +6465,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>208</v>
       </c>
@@ -6498,7 +6497,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>212</v>
       </c>
@@ -6530,7 +6529,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>217</v>
       </c>
@@ -6562,7 +6561,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>224</v>
       </c>
@@ -6594,7 +6593,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>229</v>
       </c>
@@ -6626,7 +6625,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>233</v>
       </c>
@@ -6658,7 +6657,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>237</v>
       </c>
@@ -6708,7 +6707,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>245</v>
       </c>
@@ -6758,7 +6757,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>253</v>
       </c>
@@ -6808,7 +6807,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>261</v>
       </c>
@@ -6858,7 +6857,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>270</v>
       </c>
@@ -6908,7 +6907,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>278</v>
       </c>
@@ -6958,7 +6957,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>287</v>
       </c>
@@ -6987,7 +6986,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>292</v>
       </c>
@@ -7016,7 +7015,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>297</v>
       </c>
@@ -7045,7 +7044,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>301</v>
       </c>
@@ -7095,7 +7094,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>309</v>
       </c>
@@ -7127,7 +7126,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>314</v>
       </c>
@@ -7177,7 +7176,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>323</v>
       </c>
@@ -7227,7 +7226,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>331</v>
       </c>
@@ -7259,7 +7258,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>337</v>
       </c>
@@ -7326,7 +7325,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>346</v>
       </c>
@@ -7376,7 +7375,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>353</v>
       </c>
@@ -7426,7 +7425,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>360</v>
       </c>
@@ -7476,7 +7475,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>368</v>
       </c>
@@ -7523,7 +7522,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>374</v>
       </c>
@@ -7552,7 +7551,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>379</v>
       </c>
@@ -7602,7 +7601,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>389</v>
       </c>
@@ -7652,7 +7651,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>394</v>
       </c>
@@ -7702,7 +7701,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>400</v>
       </c>
@@ -7752,7 +7751,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>406</v>
       </c>
@@ -7802,7 +7801,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>412</v>
       </c>
@@ -7852,7 +7851,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>416</v>
       </c>
@@ -7902,7 +7901,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>424</v>
       </c>
@@ -7952,7 +7951,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>432</v>
       </c>
@@ -8002,7 +8001,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>438</v>
       </c>
@@ -8102,7 +8101,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>450</v>
       </c>
@@ -8152,7 +8151,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>458</v>
       </c>
@@ -8202,7 +8201,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>466</v>
       </c>
@@ -8234,7 +8233,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>471</v>
       </c>
@@ -8269,7 +8268,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>478</v>
       </c>
@@ -8319,7 +8318,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>483</v>
       </c>
@@ -8369,7 +8368,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>491</v>
       </c>
@@ -8419,7 +8418,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>500</v>
       </c>
@@ -8469,7 +8468,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>508</v>
       </c>
@@ -8519,7 +8518,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>512</v>
       </c>
@@ -8619,7 +8618,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>525</v>
       </c>
@@ -8669,7 +8668,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>535</v>
       </c>
@@ -8719,7 +8718,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>543</v>
       </c>
@@ -8769,7 +8768,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>550</v>
       </c>
@@ -8819,7 +8818,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>558</v>
       </c>
@@ -8869,7 +8868,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>565</v>
       </c>
@@ -8919,7 +8918,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>572</v>
       </c>
@@ -8969,7 +8968,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>581</v>
       </c>
@@ -9019,7 +9018,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>588</v>
       </c>
@@ -9069,7 +9068,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>595</v>
       </c>
@@ -9119,7 +9118,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>602</v>
       </c>
@@ -9169,7 +9168,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>610</v>
       </c>
@@ -9219,7 +9218,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>617</v>
       </c>
@@ -9269,7 +9268,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>625</v>
       </c>
@@ -9319,7 +9318,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>632</v>
       </c>
@@ -9369,7 +9368,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>638</v>
       </c>
@@ -9419,7 +9418,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>644</v>
       </c>
@@ -9469,7 +9468,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>648</v>
       </c>
@@ -9869,7 +9868,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>699</v>
       </c>
@@ -9919,7 +9918,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>706</v>
       </c>
@@ -9969,7 +9968,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>713</v>
       </c>
@@ -10019,7 +10018,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>720</v>
       </c>
@@ -10069,7 +10068,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>727</v>
       </c>
@@ -10169,7 +10168,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>741</v>
       </c>
@@ -10219,7 +10218,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>748</v>
       </c>
@@ -10269,7 +10268,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>755</v>
       </c>
@@ -10319,7 +10318,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>762</v>
       </c>
@@ -10369,7 +10368,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>770</v>
       </c>
@@ -10419,7 +10418,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>777</v>
       </c>
@@ -10451,7 +10450,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>782</v>
       </c>
@@ -10501,7 +10500,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>788</v>
       </c>
@@ -10551,7 +10550,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>797</v>
       </c>
@@ -10601,7 +10600,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>805</v>
       </c>
@@ -10651,7 +10650,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>813</v>
       </c>
@@ -10701,7 +10700,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>821</v>
       </c>
@@ -10751,7 +10750,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>826</v>
       </c>
@@ -10801,7 +10800,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>831</v>
       </c>
@@ -10851,7 +10850,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>837</v>
       </c>
@@ -10901,7 +10900,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>844</v>
       </c>
@@ -10951,7 +10950,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>848</v>
       </c>
@@ -11001,7 +11000,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>855</v>
       </c>
@@ -11051,7 +11050,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>862</v>
       </c>
@@ -11101,7 +11100,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="129" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>869</v>
       </c>
@@ -11151,7 +11150,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="130" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>873</v>
       </c>
@@ -11201,7 +11200,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>877</v>
       </c>
@@ -11251,7 +11250,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>883</v>
       </c>
@@ -11301,7 +11300,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>890</v>
       </c>
@@ -11348,7 +11347,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>898</v>
       </c>
@@ -11398,7 +11397,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>906</v>
       </c>
@@ -11448,7 +11447,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>910</v>
       </c>
@@ -11498,7 +11497,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>917</v>
       </c>
@@ -11545,7 +11544,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="138" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>925</v>
       </c>
@@ -11595,7 +11594,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>930</v>
       </c>
@@ -11645,7 +11644,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>937</v>
       </c>
@@ -11695,7 +11694,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>943</v>
       </c>
@@ -11745,7 +11744,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>950</v>
       </c>
@@ -11795,7 +11794,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>956</v>
       </c>
@@ -11845,7 +11844,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>962</v>
       </c>
@@ -11945,7 +11944,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>976</v>
       </c>
@@ -11995,7 +11994,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="147" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>982</v>
       </c>
@@ -12045,7 +12044,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="148" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>990</v>
       </c>
@@ -12095,7 +12094,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>995</v>
       </c>
@@ -12127,7 +12126,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>999</v>
       </c>
@@ -12159,7 +12158,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>1003</v>
       </c>
@@ -12191,7 +12190,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>1007</v>
       </c>
@@ -12223,7 +12222,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>1011</v>
       </c>
@@ -12273,7 +12272,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>1018</v>
       </c>
@@ -12323,7 +12322,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="155" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>1024</v>
       </c>
@@ -12473,7 +12472,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>1041</v>
       </c>
@@ -12523,7 +12522,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>1048</v>
       </c>
@@ -12570,7 +12569,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>1055</v>
       </c>
@@ -12620,7 +12619,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>1060</v>
       </c>
@@ -12670,7 +12669,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>1066</v>
       </c>
@@ -12720,7 +12719,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>1074</v>
       </c>
@@ -12770,7 +12769,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>1081</v>
       </c>
@@ -12817,7 +12816,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="165" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>1087</v>
       </c>
@@ -12867,7 +12866,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="166" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>1094</v>
       </c>
@@ -12967,7 +12966,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>1108</v>
       </c>
@@ -13017,7 +13016,7 @@
         <v>1114</v>
       </c>
     </row>
-    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>1115</v>
       </c>
@@ -13067,7 +13066,7 @@
         <v>1121</v>
       </c>
     </row>
-    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>1122</v>
       </c>
@@ -13117,7 +13116,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="171" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>1128</v>
       </c>
@@ -13167,7 +13166,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>1133</v>
       </c>
@@ -13217,7 +13216,7 @@
         <v>1137</v>
       </c>
     </row>
-    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>1138</v>
       </c>
@@ -13267,7 +13266,7 @@
         <v>1144</v>
       </c>
     </row>
-    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>1145</v>
       </c>
@@ -13317,7 +13316,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>1149</v>
       </c>
@@ -13367,7 +13366,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>1156</v>
       </c>
@@ -13417,7 +13416,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>1161</v>
       </c>
@@ -13464,7 +13463,7 @@
         <v>1166</v>
       </c>
     </row>
-    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>1167</v>
       </c>
@@ -13514,7 +13513,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>1175</v>
       </c>
@@ -13564,7 +13563,7 @@
         <v>1183</v>
       </c>
     </row>
-    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>1184</v>
       </c>
@@ -13614,7 +13613,7 @@
         <v>1190</v>
       </c>
     </row>
-    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>1191</v>
       </c>
@@ -13664,7 +13663,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>1196</v>
       </c>
@@ -13714,7 +13713,7 @@
         <v>1203</v>
       </c>
     </row>
-    <row r="183" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>1204</v>
       </c>
@@ -13764,7 +13763,7 @@
         <v>1211</v>
       </c>
     </row>
-    <row r="184" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>1212</v>
       </c>
@@ -13799,7 +13798,7 @@
         <v>1217</v>
       </c>
     </row>
-    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>1218</v>
       </c>
@@ -13849,7 +13848,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>1225</v>
       </c>
@@ -13899,7 +13898,7 @@
         <v>1232</v>
       </c>
     </row>
-    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>1233</v>
       </c>
@@ -13949,7 +13948,7 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>1242</v>
       </c>
@@ -13999,7 +13998,7 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>1251</v>
       </c>
@@ -14049,7 +14048,7 @@
         <v>1256</v>
       </c>
     </row>
-    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>1257</v>
       </c>
@@ -14099,7 +14098,7 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="191" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>1264</v>
       </c>
@@ -14134,7 +14133,7 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>1270</v>
       </c>
@@ -14184,7 +14183,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>1277</v>
       </c>
@@ -14234,7 +14233,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>1284</v>
       </c>
@@ -14284,7 +14283,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>1291</v>
       </c>
@@ -14334,7 +14333,7 @@
         <v>1297</v>
       </c>
     </row>
-    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>1298</v>
       </c>
@@ -14384,7 +14383,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>1303</v>
       </c>
@@ -14434,7 +14433,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>1309</v>
       </c>
@@ -14484,7 +14483,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>1315</v>
       </c>
@@ -14534,7 +14533,7 @@
         <v>1319</v>
       </c>
     </row>
-    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>1320</v>
       </c>
@@ -14584,7 +14583,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>1324</v>
       </c>
@@ -14634,7 +14633,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>1331</v>
       </c>
@@ -14684,7 +14683,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="203" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>1336</v>
       </c>
@@ -14734,7 +14733,7 @@
         <v>1340</v>
       </c>
     </row>
-    <row r="204" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>1341</v>
       </c>
@@ -14784,7 +14783,7 @@
         <v>1348</v>
       </c>
     </row>
-    <row r="205" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>1349</v>
       </c>
@@ -14934,7 +14933,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>1368</v>
       </c>
@@ -14984,7 +14983,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>1375</v>
       </c>
@@ -15034,7 +15033,7 @@
         <v>1379</v>
       </c>
     </row>
-    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>1380</v>
       </c>
@@ -15084,7 +15083,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>1386</v>
       </c>
@@ -15134,7 +15133,7 @@
         <v>1391</v>
       </c>
     </row>
-    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>1392</v>
       </c>
@@ -15184,7 +15183,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>1399</v>
       </c>
@@ -15234,7 +15233,7 @@
         <v>1403</v>
       </c>
     </row>
-    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>1404</v>
       </c>
@@ -15284,7 +15283,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>1411</v>
       </c>
@@ -15334,7 +15333,7 @@
         <v>1415</v>
       </c>
     </row>
-    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>1416</v>
       </c>
@@ -15484,7 +15483,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>1433</v>
       </c>
@@ -15534,7 +15533,7 @@
         <v>1438</v>
       </c>
     </row>
-    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>1439</v>
       </c>
@@ -15584,7 +15583,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>1444</v>
       </c>
@@ -15634,7 +15633,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>1448</v>
       </c>
@@ -15684,7 +15683,7 @@
         <v>1454</v>
       </c>
     </row>
-    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>1455</v>
       </c>
@@ -15734,7 +15733,7 @@
         <v>1462</v>
       </c>
     </row>
-    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>1463</v>
       </c>
@@ -15784,7 +15783,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>1471</v>
       </c>
@@ -15834,7 +15833,7 @@
         <v>1478</v>
       </c>
     </row>
-    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>1479</v>
       </c>
@@ -15875,7 +15874,7 @@
         <v>1484</v>
       </c>
     </row>
-    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>1485</v>
       </c>
@@ -15916,7 +15915,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>1490</v>
       </c>
@@ -15957,7 +15956,7 @@
         <v>1493</v>
       </c>
     </row>
-    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>1494</v>
       </c>
@@ -15998,7 +15997,7 @@
         <v>1499</v>
       </c>
     </row>
-    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>1500</v>
       </c>
@@ -16039,7 +16038,7 @@
         <v>1504</v>
       </c>
     </row>
-    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>1505</v>
       </c>
@@ -16080,7 +16079,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>1511</v>
       </c>
@@ -16121,7 +16120,7 @@
         <v>1516</v>
       </c>
     </row>
-    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>1517</v>
       </c>
@@ -16162,7 +16161,7 @@
         <v>1521</v>
       </c>
     </row>
-    <row r="234" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>1522</v>
       </c>
@@ -16203,7 +16202,7 @@
         <v>1525</v>
       </c>
     </row>
-    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>1526</v>
       </c>
@@ -16244,7 +16243,7 @@
         <v>1530</v>
       </c>
     </row>
-    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>1531</v>
       </c>
@@ -16285,7 +16284,7 @@
         <v>1535</v>
       </c>
     </row>
-    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>1536</v>
       </c>
@@ -16326,7 +16325,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>1542</v>
       </c>
@@ -16367,7 +16366,7 @@
         <v>1546</v>
       </c>
     </row>
-    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>1547</v>
       </c>
@@ -16408,7 +16407,7 @@
         <v>1553</v>
       </c>
     </row>
-    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>1554</v>
       </c>
@@ -16490,7 +16489,7 @@
         <v>1562</v>
       </c>
     </row>
-    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>1563</v>
       </c>
@@ -16572,7 +16571,7 @@
         <v>1571</v>
       </c>
     </row>
-    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>1572</v>
       </c>
@@ -16613,7 +16612,7 @@
         <v>1577</v>
       </c>
     </row>
-    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>1578</v>
       </c>
@@ -16695,7 +16694,7 @@
         <v>1588</v>
       </c>
     </row>
-    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>1589</v>
       </c>
@@ -16736,7 +16735,7 @@
         <v>1594</v>
       </c>
     </row>
-    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>1595</v>
       </c>
@@ -16777,7 +16776,7 @@
         <v>1599</v>
       </c>
     </row>
-    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>1600</v>
       </c>
@@ -16818,7 +16817,7 @@
         <v>1607</v>
       </c>
     </row>
-    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>1608</v>
       </c>
@@ -16900,7 +16899,7 @@
         <v>1618</v>
       </c>
     </row>
-    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>1619</v>
       </c>
@@ -16982,7 +16981,7 @@
         <v>1631</v>
       </c>
     </row>
-    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>1632</v>
       </c>
@@ -17023,7 +17022,7 @@
         <v>1635</v>
       </c>
     </row>
-    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>1636</v>
       </c>
@@ -17105,7 +17104,7 @@
         <v>1646</v>
       </c>
     </row>
-    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>1647</v>
       </c>
@@ -17147,14 +17146,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P257" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="Equipment"/>
-        <filter val="EQUIPTMENT"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P257" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>